<commit_message>
Scene, Resource, Pooling 매니져 리펙토링 진행
</commit_message>
<xml_diff>
--- a/DesignTable/Data/Table/Tables/SceneData.xlsx
+++ b/DesignTable/Data/Table/Tables/SceneData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\ProjectT\DesignTable\Data\Table\Tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{37B80AC2-9C1E-4792-AD2C-2405E7C42780}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49937877-B6DA-477F-BD64-D3085A90477B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{4B5F7AFB-0092-4900-B3F4-0317E72BC1CA}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4B5F7AFB-0092-4900-B3F4-0317E72BC1CA}"/>
   </bookViews>
   <sheets>
     <sheet name="record" sheetId="2" r:id="rId1"/>

</xml_diff>